<commit_message>
feat: complete full migration and valuation core
</commit_message>
<xml_diff>
--- a/fixtures/sanitized/m3/cash-import-invalid.xlsx
+++ b/fixtures/sanitized/m3/cash-import-invalid.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="92">
   <si>
     <t>template_version</t>
   </si>
@@ -721,10 +721,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:10">
       <c r="A1" t="s">
         <v>6</v>
       </c>
@@ -752,8 +752,11 @@
       <c r="I1" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="2" spans="1:9">
+      <c r="J1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10">
       <c r="A2" t="s">
         <v>24</v>
       </c>
@@ -781,8 +784,11 @@
       <c r="I2" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="3" spans="1:9">
+      <c r="J2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10">
       <c r="A3" t="s">
         <v>31</v>
       </c>
@@ -810,8 +816,11 @@
       <c r="I3" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="4" spans="1:9">
+      <c r="J3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
       <c r="A4" t="s">
         <v>35</v>
       </c>
@@ -839,8 +848,11 @@
       <c r="I4" t="s">
         <v>30</v>
       </c>
-    </row>
-    <row r="5" spans="1:9">
+      <c r="J4" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10">
       <c r="A5" t="s">
         <v>40</v>
       </c>
@@ -864,6 +876,9 @@
       </c>
       <c r="H5" t="s">
         <v>29</v>
+      </c>
+      <c r="J5" t="s">
+        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: preserve imported fx overrides
</commit_message>
<xml_diff>
--- a/fixtures/sanitized/m3/cash-import-invalid.xlsx
+++ b/fixtures/sanitized/m3/cash-import-invalid.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="92">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="104">
   <si>
     <t>template_version</t>
   </si>
@@ -32,7 +32,7 @@
     <t>ui_locale</t>
   </si>
   <si>
-    <t>ledgerkit-workbook-v1.3</t>
+    <t>ledgerkit-workbook-v1.4</t>
   </si>
   <si>
     <t>CNY</t>
@@ -248,6 +248,24 @@
     <t>display_label</t>
   </si>
   <si>
+    <t>fx_override_currency</t>
+  </si>
+  <si>
+    <t>fx_override_value</t>
+  </si>
+  <si>
+    <t>fx_override_reason</t>
+  </si>
+  <si>
+    <t>fee_fx_override_currency</t>
+  </si>
+  <si>
+    <t>fee_fx_override_value</t>
+  </si>
+  <si>
+    <t>fee_fx_override_reason</t>
+  </si>
+  <si>
     <t>2026-02-01</t>
   </si>
   <si>
@@ -285,6 +303,24 @@
   </si>
   <si>
     <t>to_amount</t>
+  </si>
+  <si>
+    <t>from_fx_override_currency</t>
+  </si>
+  <si>
+    <t>from_fx_override_value</t>
+  </si>
+  <si>
+    <t>from_fx_override_reason</t>
+  </si>
+  <si>
+    <t>to_fx_override_currency</t>
+  </si>
+  <si>
+    <t>to_fx_override_value</t>
+  </si>
+  <si>
+    <t>to_fx_override_reason</t>
   </si>
   <si>
     <t>2026-02-04</t>
@@ -985,10 +1021,10 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N3"/>
+  <dimension ref="A1:T3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:14">
+    <row r="1" spans="1:20">
       <c r="A1" t="s">
         <v>62</v>
       </c>
@@ -1031,16 +1067,34 @@
       <c r="N1" t="s">
         <v>74</v>
       </c>
-    </row>
-    <row r="2" spans="1:14">
+      <c r="O1" t="s">
+        <v>75</v>
+      </c>
+      <c r="P1" t="s">
+        <v>76</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>77</v>
+      </c>
+      <c r="R1" t="s">
+        <v>78</v>
+      </c>
+      <c r="S1" t="s">
+        <v>79</v>
+      </c>
+      <c r="T1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="2" spans="1:20">
       <c r="A2" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="B2" t="s">
         <v>46</v>
       </c>
       <c r="C2" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="D2" t="s">
         <v>24</v>
@@ -1053,10 +1107,10 @@
         <v>25</v>
       </c>
       <c r="G2" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="H2" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="I2" t="s">
         <v>53</v>
@@ -1074,18 +1128,18 @@
         <v>Income item</v>
       </c>
     </row>
-    <row r="3" spans="1:14">
+    <row r="3" spans="1:20">
       <c r="A3" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="B3" t="s">
         <v>46</v>
       </c>
       <c r="C3" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="D3" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="E3" t="s">
         <v>50</v>
@@ -1105,10 +1159,10 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:I2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:9">
       <c r="A1" t="s">
         <v>62</v>
       </c>
@@ -1116,10 +1170,10 @@
         <v>63</v>
       </c>
       <c r="C1" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="D1" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="E1" t="s">
         <v>67</v>
@@ -1127,10 +1181,19 @@
       <c r="F1" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="2" spans="1:6">
+      <c r="G1" t="s">
+        <v>75</v>
+      </c>
+      <c r="H1" t="s">
+        <v>76</v>
+      </c>
+      <c r="I1" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="B2" t="s">
         <v>46</v>
@@ -1145,7 +1208,7 @@
         <v>39</v>
       </c>
       <c r="F2" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
     </row>
   </sheetData>
@@ -1155,10 +1218,10 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I2"/>
+  <dimension ref="A1:R2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:18">
       <c r="A1" t="s">
         <v>62</v>
       </c>
@@ -1166,16 +1229,16 @@
         <v>63</v>
       </c>
       <c r="C1" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="D1" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="E1" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="F1" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="G1" t="s">
         <v>70</v>
@@ -1186,10 +1249,37 @@
       <c r="I1" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="2" spans="1:9">
+      <c r="J1" t="s">
+        <v>94</v>
+      </c>
+      <c r="K1" t="s">
+        <v>95</v>
+      </c>
+      <c r="L1" t="s">
+        <v>96</v>
+      </c>
+      <c r="M1" t="s">
+        <v>97</v>
+      </c>
+      <c r="N1" t="s">
+        <v>98</v>
+      </c>
+      <c r="O1" t="s">
+        <v>99</v>
+      </c>
+      <c r="P1" t="s">
+        <v>78</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>79</v>
+      </c>
+      <c r="R1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18">
       <c r="A2" t="s">
-        <v>88</v>
+        <v>100</v>
       </c>
       <c r="B2" t="s">
         <v>46</v>
@@ -1201,10 +1291,10 @@
         <v>24</v>
       </c>
       <c r="E2" t="s">
-        <v>89</v>
+        <v>101</v>
       </c>
       <c r="F2" t="s">
-        <v>90</v>
+        <v>102</v>
       </c>
       <c r="G2" t="s">
         <v>35</v>
@@ -1213,7 +1303,7 @@
         <v>46</v>
       </c>
       <c r="I2" t="s">
-        <v>91</v>
+        <v>103</v>
       </c>
     </row>
   </sheetData>

</xml_diff>